<commit_message>
Updated KEN_grids_kan model - 2025-11-30 00:12
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A35A3732-9688-4E4F-8CE5-C93CB8CBAF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E35234C3-1831-49DC-A5BC-CDE6C5582FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="12683" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="56" r:id="rId1"/>
@@ -26772,7 +26772,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D44F1D88-7831-44E2-A62B-670B13143937}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A6653B3-B6BA-4C9B-92CE-343DD10996AC}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -28765,7 +28765,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76B5B4EE-D5D4-40ED-966E-019A8FA63D01}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B3EACDE-3047-4F5C-9922-7BBFCCF37CBD}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-05 16:23
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{305B0C81-E078-41DA-B4F6-6B2E8A2B8917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{797ABAB0-E951-482E-A97F-E81AF7B59DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27500,7 +27500,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA5F71A1-F981-44BD-88AB-E92D70CA5AEE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3346AFDC-2F12-4A5B-99D2-C76778EF1618}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29493,7 +29493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC327CE3-F1BA-4FE9-B827-C4D39A5F5749}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AECFEC06-5404-46D2-A42D-26ABA8787A20}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-05 21:29
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{797ABAB0-E951-482E-A97F-E81AF7B59DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{43569429-0E1B-4458-8B0D-4F65FBF6E817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27500,7 +27500,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3346AFDC-2F12-4A5B-99D2-C76778EF1618}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47BC2CF0-8CCF-4CF3-A638-FC8BDD053804}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29493,7 +29493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AECFEC06-5404-46D2-A42D-26ABA8787A20}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85B45987-5F1C-4935-93E7-30FF8BBF1F37}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-06 12:50
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43569429-0E1B-4458-8B0D-4F65FBF6E817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15EA102-4E1F-462D-9D60-F368CCD7EF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27500,7 +27500,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47BC2CF0-8CCF-4CF3-A638-FC8BDD053804}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DACCF738-423D-4DCD-AF84-268C07DD0631}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29493,7 +29493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85B45987-5F1C-4935-93E7-30FF8BBF1F37}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB563BF1-3718-493A-ACD0-4A7CC80CF879}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-06 14:21
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C15EA102-4E1F-462D-9D60-F368CCD7EF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC6DE3E8-846F-47F0-82AF-A8E1156E6CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27500,7 +27500,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DACCF738-423D-4DCD-AF84-268C07DD0631}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55BF93F6-3EC4-4A1E-BD84-F8A2F87F9616}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -29493,7 +29493,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB563BF1-3718-493A-ACD0-4A7CC80CF879}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3DDCB97-6523-4CB5-9772-E1B58D52B122}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-12 13:51
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B44FBC2B-2AE8-4430-80D7-82EE523AF2D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{41591F16-1751-4FE6-AD5C-762833C9BE7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2938,7 +2938,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{883A003A-4038-4F1D-A29B-FE1B73141729}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F2058D6-66E0-4533-9DD7-F8466D8A3739}">
   <dimension ref="B9:H110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -24734,7 +24734,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC4179E5-6413-49BA-98C8-549DCF46F0FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0DA8948-F4E2-4038-92E6-045D87E9120A}">
   <dimension ref="B9:L110"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>